<commit_message>
Address late CodeRabbit review on PR #17
- CI: actions/checkout with persist-credentials: false in both jobs, so
  npm and pip lifecycle scripts can't read the checkout token.
- ADR-003, ADR-004 and the back-end README: whole-hostname Cloudflare
  Access is stated as a deployment requirement. The Basic gate is
  verified in production; Access denial of unlisted emails is still on
  the remote checklist.
- README: "proposed V1 workflow" while ADR-002 is Proposed.
- Workbook: cpu_ms records the single production episode (0-4 ms per
  request, not a load test) and keeps 5 ms as the planning value.

Tests: make test (142); pytest data_pipelines data_foundation/tests
evals/intake intake_agent (163); compileall; ng test (17); front-end
build; back-end unit (28) and local-D1 integration (13).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/Costs/Intake/INTAKE_COST_ESTIMATE.xlsx
+++ b/Docs/Costs/Intake/INTAKE_COST_ESTIMATE.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>D1 queries, rows and stored bytes come from local tests (back-end/test/integration/budget.test.js; SQLite with the Worker migrations). Worker CPU is not measured yet.</t>
+          <t>D1 queries, rows and stored bytes come from local tests (back-end/test/integration/budget.test.js; SQLite with the Worker migrations). Worker CPU was observed once in production (one episode, 0-4 ms per request, against the 10 ms Free limit). That was not a load test, so the model keeps 5 ms as a conservative planning value.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Worker CPU per request</t>
+          <t>Worker CPU per request (planning value)</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Not measured; read the real value from Workers analytics after deploy</t>
+          <t>Conservative planning assumption. One production episode on 2026-09-29 (Workers Logs, 13 invocations) showed 0-4 ms per request; that is a single sample, not a load test. Free limit: 10 ms</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>assumption; single-episode observation 0-4 ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align the cost workbook with the 2026-10-20 shutdown
Final pre-push review: the workbook ADR-004 cites still used a 32-day
window to 2026-10-31. The builder now uses 22 days to 2026-10-20, says it
models the legacy /cases flow (guided capacity is in ADR-004 section 2),
and the .xlsx is regenerated. ADR-004 also says the 400 MB trigger arrives
at about the end of the window (22.2 days), not inside it.

Tests: build_workbook.py --print runs; no 2026-10-31 left in the workbook;
pytest evals data_profiles/findings (114 passed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/Costs/Intake/INTAKE_COST_ESTIMATE.xlsx
+++ b/Docs/Costs/Intake/INTAKE_COST_ESTIMATE.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Run the intake service on Cloudflare Workers + D1 Free through 2026-10-31. Move to Workers Paid ($5/month) if any daily Free limit stays above 70% for 3 days.</t>
+          <t>Run the intake service on Cloudflare Workers + D1 Free through 2026-10-20. Move to Workers Paid ($5/month) if any daily Free limit stays above 70% for 3 days. This workbook models the legacy /cases flow; the guided flow's capacity (about 2,380 episodes a day) is in ADR-004 section 2.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 to 2026-10-31. Finalists are announced on 2026-10-15.</t>
+          <t>2026-09-29 to 2026-10-20. Finalists are announced on 2026-10-15; everything online is shut down after 2026-10-20.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 to 2026-10-31</t>
+          <t>2026-09-29 to 2026-10-20 (shutdown after 2026-10-20, ADR-004)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Cases stored by 2026-10-31 (MB, typical)</t>
+          <t>Cases stored by 2026-10-20 (MB, typical)</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Share of 500 MB by 2026-10-31 (2,000-char cases)</t>
+          <t>Share of 500 MB by 2026-10-20 (2,000-char cases)</t>
         </is>
       </c>
     </row>

</xml_diff>